<commit_message>
Implémentation des sections CDA de la partie corps (#117)
* MAJ-sections-CDA (#113)

* Sections cda (#116)

* MAJ des profils fsh des sections

* Renommage du profil FRActProcedureDocument (#112)

* MAJ des ids des profils sections CDA

* MAJ ressources CDA section

* MAJ sections FR-Resultats

* Correction suite à workflow failed

* Correction suite à workflow failed

* Mise à jour des sections (#118)

* MAJ des profils fsh des sections

* MAJ des ids des profils sections CDA

* MAJ ressources CDA section

* MAJ sections FR-Resultats

* Mise à jour des ids des sections + cardinalités des attributs du code

* Mise à jour des sections CDA (#119)

---------

Co-authored-by: Haoura <121106042+Haoura@users.noreply.github.com> 1d7b7e95418a31a06814d65c3f5fe5ee328ec582
</commit_message>
<xml_diff>
--- a/main/ig/FRSectionExposureRadiationLMCDAFHIR.xlsx
+++ b/main/ig/FRSectionExposureRadiationLMCDAFHIR.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="60">
   <si>
     <t>Property</t>
   </si>
@@ -55,7 +55,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-04-15T15:41:19+00:00</t>
+    <t>2026-04-20T15:11:12+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -157,10 +157,13 @@
     <t>FRLMExpositionRadiations.entree.observationGrossesse</t>
   </si>
   <si>
-    <t>FRCDADICOMExpositionAuxRadiations.entry:frDICOMObservation</t>
+    <t>FRCDADICOMExpositionAuxRadiations.entry:frDicomObservationGrossesse</t>
   </si>
   <si>
     <t>FRLMExpositionRadiations.entree.observationIndication</t>
+  </si>
+  <si>
+    <t>FRCDADICOMExpositionAuxRadiations.entry:frDicomObservationIndication</t>
   </si>
   <si>
     <t>https://interop.esante.gouv.fr/ig/document/core/StructureDefinition/fr-composition-document</t>
@@ -592,7 +595,7 @@
         <v>32</v>
       </c>
       <c r="D11" t="s" s="2">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E11" s="2"/>
     </row>
@@ -634,7 +637,7 @@
         <v>29</v>
       </c>
       <c r="D2" t="s" s="2">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E2" t="s" s="2">
         <v>29</v>
@@ -649,7 +652,7 @@
         <v>32</v>
       </c>
       <c r="D3" t="s" s="2">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E3" s="2"/>
     </row>
@@ -662,7 +665,7 @@
         <v>32</v>
       </c>
       <c r="D4" t="s" s="2">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E4" s="2"/>
     </row>
@@ -675,7 +678,7 @@
         <v>32</v>
       </c>
       <c r="D5" t="s" s="2">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E5" s="2"/>
     </row>
@@ -688,7 +691,7 @@
         <v>32</v>
       </c>
       <c r="D6" t="s" s="2">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E6" s="2"/>
     </row>
@@ -701,7 +704,7 @@
         <v>32</v>
       </c>
       <c r="D7" t="s" s="2">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E7" s="2"/>
     </row>
@@ -714,7 +717,7 @@
         <v>32</v>
       </c>
       <c r="D8" t="s" s="2">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E8" s="2"/>
     </row>
@@ -727,7 +730,7 @@
         <v>32</v>
       </c>
       <c r="D9" t="s" s="2">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E9" s="2"/>
     </row>
@@ -740,20 +743,20 @@
         <v>32</v>
       </c>
       <c r="D10" t="s" s="2">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E10" s="2"/>
     </row>
     <row r="11">
       <c r="A11" t="s" s="2">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" t="s" s="2">
         <v>32</v>
       </c>
       <c r="D11" t="s" s="2">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E11" s="2"/>
     </row>

</xml_diff>